<commit_message>
corrected reference in combined processing, re-rendered
</commit_message>
<xml_diff>
--- a/data/combined/processed/codebook_participantlevel.xlsx
+++ b/data/combined/processed/codebook_participantlevel.xlsx
@@ -384,7 +384,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>Participant identifier (character; unique within source).</t>
         </is>
       </c>
     </row>
@@ -401,7 +401,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>Scale name (or attitude-object name).</t>
         </is>
       </c>
     </row>
@@ -418,7 +418,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>Dataset / contributing-sample label.</t>
         </is>
       </c>
     </row>
@@ -435,7 +435,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>Variable type: 'trait' or 'attitude'.</t>
         </is>
       </c>
     </row>
@@ -452,7 +452,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>Theoretical minimum of the item response scale.</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>Theoretical maximum of the item response scale.</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>Participant's mean answered item response for this scale.</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>Full-scale item count (median answered items per participant for this scale, source).</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>Mean-projected sum score: mean_response * n_items (= raw sum for complete responders).</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>Sum score rescaled to [0, 1] as a proportion of the scale's logical range (POMP).</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>Number of participants with a score for this (scale, source); used by the SK transform.</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>Smithson-Verkuilen transform of pomp_sumscore: (y*(n-1) + 0.5)/n, offset off the 0/1 limits.</t>
         </is>
       </c>
     </row>

</xml_diff>